<commit_message>
Inventario: estado Activo, Holstery y consumibles ring/fork
Unifica Comprado/Ya tengo a Activo. Anade Holstery, Railer, MTO, guantes 400V y kits ring/fork Amazon.
</commit_message>
<xml_diff>
--- a/Herramientas/inventario/Arsenal_Multioficio_2026.xlsx
+++ b/Herramientas/inventario/Arsenal_Multioficio_2026.xlsx
@@ -13,9 +13,9 @@
     <sheet name="Consumibles" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inventario'!$A$4:$K$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inventario'!$A$4:$K$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pendientes'!$A$4:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Consumibles'!$A$4:$L$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Consumibles'!$A$4:$L$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -110,7 +110,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -135,11 +135,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F3F4F6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -224,12 +219,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -269,49 +264,58 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -323,6 +327,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -337,12 +347,6 @@
     <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -353,18 +357,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -733,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -775,7 +767,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -790,7 +782,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -801,11 +793,11 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Estado: Ya tengo (lineas)</t>
+          <t>Estado: Activo (lineas)</t>
         </is>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Inventario!I5:I46,"Ya tengo")</f>
+        <f>COUNTIF(Inventario!I5:I52,"Activo")</f>
         <v/>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -817,12 +809,11 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Estado: Comprado (lineas)</t>
-        </is>
-      </c>
-      <c r="B8" s="5">
-        <f>COUNTIF(Inventario!I5:I46,"Comprado")</f>
-        <v/>
+          <t>Pendientes de compra</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -833,11 +824,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Pendientes de compra</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>6</v>
+          <t>Costo estimado pendientes (CRC)</t>
+        </is>
+      </c>
+      <c r="B9" s="6">
+        <f>SUM(Pendientes!F5:F10)</f>
+        <v/>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -848,12 +840,11 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Costo estimado pendientes (CRC)</t>
-        </is>
-      </c>
-      <c r="B10" s="6">
-        <f>SUM(Pendientes!F5:F10)</f>
-        <v/>
+          <t>Lineas de consumibles (kits)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>14</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
@@ -864,11 +855,12 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Lineas de consumibles (kits)</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>12</v>
+          <t>Consumibles a reponer</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>COUNTIF(Consumibles!J5:J18,"Reponer")</f>
+        <v/>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
@@ -876,35 +868,31 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Consumibles a reponer</t>
-        </is>
-      </c>
-      <c r="B12" s="5">
-        <f>COUNTIF(Consumibles!J5:J16,"Reponer")</f>
-        <v/>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Esquema de codigos (por LINEA)</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Esquema de codigos (por LINEA)</t>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Inventario: MARCA-FAMILIA-###  (ej. MW-M12-001, KL-ELC-003, MW-M12-BAT-001)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Inventario: MARCA-FAMILIA-###  (ej. MW-M12-001, KL-ELC-003, MW-M12-BAT-001)</t>
+          <t>Un codigo = una linea, no una unidad fisica. Cantidad en columna aparte.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Un codigo = una linea, no una unidad fisica. Cantidad en columna aparte.</t>
+          <t>Estado inventario: Activo (en arsenal). Baja/Prestado opcionales. Pendientes en hoja aparte.</t>
         </is>
       </c>
     </row>
@@ -1006,154 +994,210 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Huepar</t>
+          <t>Holstery</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>https://huepar.com/</t>
+          <t>https://holstery.com/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>LEXIVON</t>
+          <t>Huepar</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>https://www.lexivon.com/</t>
+          <t>https://huepar.com/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
+          <t>LEXIVON</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>https://www.lexivon.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
           <t>Skil</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>https://www.skil.com/</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Lineas por marca</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Lineas</t>
         </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>Antive</t>
-        </is>
-      </c>
-      <c r="B34" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A34)</f>
-        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>Franklin</t>
+          <t>Antive</t>
         </is>
       </c>
       <c r="B35" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A35)</f>
+        <f>COUNTIF(Inventario!C5:C52,A35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Huepar</t>
+          <t>Franklin</t>
         </is>
       </c>
       <c r="B36" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A36)</f>
+        <f>COUNTIF(Inventario!C5:C52,A36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>Klein</t>
+          <t>Holstery</t>
         </is>
       </c>
       <c r="B37" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A37)</f>
+        <f>COUNTIF(Inventario!C5:C52,A37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Knipex</t>
+          <t>Huepar</t>
         </is>
       </c>
       <c r="B38" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A38)</f>
+        <f>COUNTIF(Inventario!C5:C52,A38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>LEXIVON</t>
+          <t>Klein</t>
         </is>
       </c>
       <c r="B39" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A39)</f>
+        <f>COUNTIF(Inventario!C5:C52,A39)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Knipex</t>
         </is>
       </c>
       <c r="B40" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A40)</f>
+        <f>COUNTIF(Inventario!C5:C52,A40)</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>Skil</t>
+          <t>LEXIVON</t>
         </is>
       </c>
       <c r="B41" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A41)</f>
+        <f>COUNTIF(Inventario!C5:C52,A41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
+          <t>MTO</t>
+        </is>
+      </c>
+      <c r="B42" s="11">
+        <f>COUNTIF(Inventario!C5:C52,A42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>Milwaukee</t>
+        </is>
+      </c>
+      <c r="B43" s="11">
+        <f>COUNTIF(Inventario!C5:C52,A43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Railer</t>
+        </is>
+      </c>
+      <c r="B44" s="11">
+        <f>COUNTIF(Inventario!C5:C52,A44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Skil</t>
+        </is>
+      </c>
+      <c r="B45" s="11">
+        <f>COUNTIF(Inventario!C5:C52,A45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
           <t>Wera</t>
         </is>
       </c>
-      <c r="B42" s="11">
-        <f>COUNTIF(Inventario!C5:C46,A42)</f>
+      <c r="B46" s="11">
+        <f>COUNTIF(Inventario!C5:C52,A46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>Youneedthat</t>
+        </is>
+      </c>
+      <c r="B47" s="11">
+        <f>COUNTIF(Inventario!C5:C52,A47)</f>
         <v/>
       </c>
     </row>
@@ -1169,6 +1213,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1180,7 +1225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1220,7 +1265,7 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G2" s="12" t="inlineStr">
         <is>
@@ -1228,7 +1273,7 @@
         </is>
       </c>
       <c r="H2" s="3" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -1334,7 +1379,7 @@
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J5" s="18" t="inlineStr">
@@ -1385,9 +1430,9 @@
       <c r="H6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J6" s="18" t="inlineStr">
@@ -1438,9 +1483,9 @@
       <c r="H7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J7" s="18" t="inlineStr">
@@ -1491,9 +1536,9 @@
       <c r="H8" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J8" s="18" t="inlineStr">
@@ -1546,7 +1591,7 @@
       </c>
       <c r="I9" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J9" s="18" t="inlineStr">
@@ -1597,9 +1642,9 @@
       <c r="H10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J10" s="18" t="inlineStr">
@@ -1650,9 +1695,9 @@
       <c r="H11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I11" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J11" s="18" t="inlineStr">
@@ -1703,9 +1748,9 @@
       <c r="H12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J12" s="18" t="inlineStr">
@@ -1756,9 +1801,9 @@
       <c r="H13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J13" s="18" t="inlineStr">
@@ -1809,9 +1854,9 @@
       <c r="H14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J14" s="18" t="inlineStr">
@@ -1862,9 +1907,9 @@
       <c r="H15" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I15" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J15" s="18" t="inlineStr">
@@ -1915,9 +1960,9 @@
       <c r="H16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J16" s="18" t="inlineStr">
@@ -1968,9 +2013,9 @@
       <c r="H17" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I17" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J17" s="18" t="inlineStr">
@@ -2021,9 +2066,9 @@
       <c r="H18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J18" s="18" t="inlineStr">
@@ -2074,9 +2119,9 @@
       <c r="H19" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I19" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J19" s="18" t="inlineStr">
@@ -2127,9 +2172,9 @@
       <c r="H20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J20" s="18" t="inlineStr">
@@ -2182,7 +2227,7 @@
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J21" s="18" t="inlineStr">
@@ -2235,7 +2280,7 @@
       </c>
       <c r="I22" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J22" s="18" t="inlineStr">
@@ -2288,7 +2333,7 @@
       </c>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J23" s="18" t="inlineStr">
@@ -2339,9 +2384,9 @@
       <c r="H24" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I24" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J24" s="18" t="inlineStr">
@@ -2392,9 +2437,9 @@
       <c r="H25" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I25" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J25" s="18" t="inlineStr">
@@ -2445,9 +2490,9 @@
       <c r="H26" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I26" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I26" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J26" s="18" t="inlineStr">
@@ -2498,9 +2543,9 @@
       <c r="H27" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I27" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J27" s="18" t="inlineStr">
@@ -2551,9 +2596,9 @@
       <c r="H28" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I28" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I28" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J28" s="18" t="inlineStr">
@@ -2604,9 +2649,9 @@
       <c r="H29" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I29" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I29" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J29" s="18" t="inlineStr">
@@ -2659,7 +2704,7 @@
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J30" s="18" t="inlineStr">
@@ -2712,7 +2757,7 @@
       </c>
       <c r="I31" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J31" s="18" t="inlineStr">
@@ -2763,9 +2808,9 @@
       <c r="H32" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I32" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I32" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J32" s="18" t="inlineStr">
@@ -2816,9 +2861,9 @@
       <c r="H33" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I33" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J33" s="18" t="inlineStr">
@@ -2869,9 +2914,9 @@
       <c r="H34" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="I34" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I34" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J34" s="18" t="inlineStr">
@@ -2924,7 +2969,7 @@
       </c>
       <c r="I35" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J35" s="18" t="inlineStr">
@@ -2977,7 +3022,7 @@
       </c>
       <c r="I36" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J36" s="18" t="inlineStr">
@@ -3030,7 +3075,7 @@
       </c>
       <c r="I37" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J37" s="18" t="inlineStr">
@@ -3083,7 +3128,7 @@
       </c>
       <c r="I38" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J38" s="18" t="inlineStr">
@@ -3103,50 +3148,50 @@
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>SK-ELC-001</t>
+          <t>HO-ORG-001</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Skil</t>
+          <t>Holstery</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Herramienta</t>
+          <t>Organizacion</t>
         </is>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>Electrica</t>
+          <t>Organizacion</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>Martillo Automatico</t>
+          <t>ModPouch Clip-On Modular Tool Pouch (Standard)</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr">
         <is>
-          <t>AH6552A-00</t>
+          <t>ModPouch</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I39" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I39" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J39" s="18" t="inlineStr">
         <is>
-          <t>Ver en Skil</t>
+          <t>Ver en Holstery</t>
         </is>
       </c>
       <c r="K39" s="19" t="inlineStr">
         <is>
-          <t>https://www.skil.com/search?q=AH6552A</t>
+          <t>https://holstery.com/products/mod-pouch-clip-on-modular-tool-pouch</t>
         </is>
       </c>
     </row>
@@ -3156,50 +3201,50 @@
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>AN-ELC-001</t>
+          <t>HO-ORG-002</t>
         </is>
       </c>
       <c r="C40" s="20" t="inlineStr">
         <is>
-          <t>Antive</t>
+          <t>Holstery</t>
         </is>
       </c>
       <c r="D40" s="20" t="inlineStr">
         <is>
-          <t>Herramienta</t>
+          <t>Organizacion</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
         <is>
-          <t>Electrica</t>
+          <t>Organizacion</t>
         </is>
       </c>
       <c r="F40" s="21" t="inlineStr">
         <is>
-          <t>Tijeras Electricas Inalambricas</t>
+          <t>DriverMaster Clip-On Drill Holster</t>
         </is>
       </c>
       <c r="G40" s="20" t="inlineStr">
         <is>
-          <t>E-S01</t>
+          <t>DriverMaster</t>
         </is>
       </c>
       <c r="H40" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I40" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I40" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J40" s="18" t="inlineStr">
         <is>
-          <t>Ver en Antive</t>
+          <t>Ver en Holstery</t>
         </is>
       </c>
       <c r="K40" s="19" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/s?k=Antive+E-S01+electric+scissors</t>
+          <t>https://holstery.com/products/drivermaster-v2-clip-on-drill-holster</t>
         </is>
       </c>
     </row>
@@ -3209,50 +3254,50 @@
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>HP-PRE-001</t>
+          <t>HO-ORG-003</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Huepar</t>
+          <t>Holstery</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Herramienta</t>
+          <t>Organizacion</t>
         </is>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>Precision</t>
+          <t>Organizacion</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>Nivel Laser Verde Cross-Line</t>
+          <t>MagMaster Magnetic Tool and Hardware Holder</t>
         </is>
       </c>
       <c r="G41" s="11" t="inlineStr">
         <is>
-          <t>BOX-1G</t>
+          <t>MagMaster V2</t>
         </is>
       </c>
       <c r="H41" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I41" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I41" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J41" s="18" t="inlineStr">
         <is>
-          <t>Ver en Huepar</t>
+          <t>Ver en Holstery</t>
         </is>
       </c>
       <c r="K41" s="19" t="inlineStr">
         <is>
-          <t>https://huepar.com/products/huepar-box1g-laser-level</t>
+          <t>https://holstery.com/products/magmaster-v2-magnetic-tool-and-hardware-holder</t>
         </is>
       </c>
     </row>
@@ -3262,50 +3307,50 @@
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>FR-PRE-001</t>
+          <t>RA-ORG-001</t>
         </is>
       </c>
       <c r="C42" s="20" t="inlineStr">
         <is>
-          <t>Franklin</t>
+          <t>Railer</t>
         </is>
       </c>
       <c r="D42" s="20" t="inlineStr">
         <is>
-          <t>Herramienta</t>
+          <t>Organizacion</t>
         </is>
       </c>
       <c r="E42" s="21" t="inlineStr">
         <is>
-          <t>Precision</t>
+          <t>Organizacion</t>
         </is>
       </c>
       <c r="F42" s="21" t="inlineStr">
         <is>
-          <t>Nivel Digital Electronico</t>
+          <t>Bitrail 20-hole bit holder set (2 pc) + carabiners</t>
         </is>
       </c>
       <c r="G42" s="20" t="inlineStr">
         <is>
-          <t>iA12</t>
+          <t>RB2BKORC</t>
         </is>
       </c>
       <c r="H42" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+        <v>2</v>
+      </c>
+      <c r="I42" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J42" s="18" t="inlineStr">
         <is>
-          <t>Ver en Franklin</t>
+          <t>Ver en Railer</t>
         </is>
       </c>
       <c r="K42" s="19" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/s?k=Franklin+Sensors+iA12</t>
+          <t>https://www.amazon.com/dp/B0CNDY32SX</t>
         </is>
       </c>
     </row>
@@ -3315,12 +3360,12 @@
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>LX-SLD-001</t>
+          <t>SK-ELC-001</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>LEXIVON</t>
+          <t>Skil</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
@@ -3330,35 +3375,35 @@
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>Soldadura</t>
+          <t>Electrica</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>Soldador de Butano 7 puntas</t>
+          <t>Martillo Automatico</t>
         </is>
       </c>
       <c r="G43" s="11" t="inlineStr">
         <is>
-          <t>LX-770</t>
+          <t>AH6552A-00</t>
         </is>
       </c>
       <c r="H43" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I43" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I43" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J43" s="18" t="inlineStr">
         <is>
-          <t>Ver en LEXIVON</t>
+          <t>Ver en Skil</t>
         </is>
       </c>
       <c r="K43" s="19" t="inlineStr">
         <is>
-          <t>https://www.lexivon.com/products/lx-770</t>
+          <t>https://www.skil.com/search?q=AH6552A</t>
         </is>
       </c>
     </row>
@@ -3368,50 +3413,50 @@
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>MW-SEG-001</t>
+          <t>AN-ELC-001</t>
         </is>
       </c>
       <c r="C44" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Antive</t>
         </is>
       </c>
       <c r="D44" s="20" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Herramienta</t>
         </is>
       </c>
       <c r="E44" s="21" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Electrica</t>
         </is>
       </c>
       <c r="F44" s="21" t="inlineStr">
         <is>
-          <t>Lentes de seguridad</t>
+          <t>Tijeras Electricas Inalambricas</t>
         </is>
       </c>
       <c r="G44" s="20" t="inlineStr">
         <is>
-          <t>48-73-2013</t>
+          <t>E-S01</t>
         </is>
       </c>
       <c r="H44" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I44" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I44" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J44" s="18" t="inlineStr">
         <is>
-          <t>Ver en Milwaukee</t>
+          <t>Ver en Antive</t>
         </is>
       </c>
       <c r="K44" s="19" t="inlineStr">
         <is>
-          <t>https://www.milwaukeetool.com/Search?q=48-73-2013</t>
+          <t>https://www.amazon.com/s?k=Antive+E-S01+electric+scissors</t>
         </is>
       </c>
     </row>
@@ -3421,50 +3466,50 @@
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>MW-SEG-002</t>
+          <t>HP-PRE-001</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Huepar</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Herramienta</t>
         </is>
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Precision</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>Guantes PACKOUT Cut Level 1 Smartswipe</t>
+          <t>Nivel Laser Verde Cross-Line</t>
         </is>
       </c>
       <c r="G45" s="11" t="inlineStr">
         <is>
-          <t>48-73-2013</t>
+          <t>BOX-1G</t>
         </is>
       </c>
       <c r="H45" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="I45" s="22" t="inlineStr">
-        <is>
-          <t>Ya tengo</t>
+      <c r="I45" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J45" s="18" t="inlineStr">
         <is>
-          <t>Ver en Milwaukee</t>
+          <t>Ver en Huepar</t>
         </is>
       </c>
       <c r="K45" s="19" t="inlineStr">
         <is>
-          <t>https://www.milwaukeetool.com/Search?q=PACKOUT+Cut+Level+Smartswipe+gloves</t>
+          <t>https://huepar.com/products/huepar-box1g-laser-level</t>
         </is>
       </c>
     </row>
@@ -3474,32 +3519,32 @@
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>MW-ACC-001</t>
+          <t>FR-PRE-001</t>
         </is>
       </c>
       <c r="C46" s="20" t="inlineStr">
         <is>
-          <t>Milwaukee</t>
+          <t>Franklin</t>
         </is>
       </c>
       <c r="D46" s="20" t="inlineStr">
         <is>
-          <t>Accesorio</t>
+          <t>Herramienta</t>
         </is>
       </c>
       <c r="E46" s="21" t="inlineStr">
         <is>
-          <t>Accesorio</t>
+          <t>Precision</t>
         </is>
       </c>
       <c r="F46" s="21" t="inlineStr">
         <is>
-          <t>Juego de 3 hojas para Multi-Tool</t>
+          <t>Nivel Digital Electronico</t>
         </is>
       </c>
       <c r="G46" s="20" t="inlineStr">
         <is>
-          <t>49-10-9001</t>
+          <t>iA12</t>
         </is>
       </c>
       <c r="H46" s="11" t="n">
@@ -3507,29 +3552,347 @@
       </c>
       <c r="I46" s="17" t="inlineStr">
         <is>
-          <t>Comprado</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="J46" s="18" t="inlineStr">
         <is>
+          <t>Ver en Franklin</t>
+        </is>
+      </c>
+      <c r="K46" s="19" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/s?k=Franklin+Sensors+iA12</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>LX-SLD-001</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>LEXIVON</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>Herramienta</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>Soldadura</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>Soldador de Butano 7 puntas</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>LX-770</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="J47" s="18" t="inlineStr">
+        <is>
+          <t>Ver en LEXIVON</t>
+        </is>
+      </c>
+      <c r="K47" s="19" t="inlineStr">
+        <is>
+          <t>https://www.lexivon.com/products/lx-770</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>MW-SEG-001</t>
+        </is>
+      </c>
+      <c r="C48" s="20" t="inlineStr">
+        <is>
+          <t>Milwaukee</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="E48" s="21" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="F48" s="21" t="inlineStr">
+        <is>
+          <t>Lentes de seguridad</t>
+        </is>
+      </c>
+      <c r="G48" s="20" t="inlineStr">
+        <is>
+          <t>48-73-2013</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I48" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="J48" s="18" t="inlineStr">
+        <is>
           <t>Ver en Milwaukee</t>
         </is>
       </c>
-      <c r="K46" s="19" t="inlineStr">
+      <c r="K48" s="19" t="inlineStr">
+        <is>
+          <t>https://www.milwaukeetool.com/Search?q=48-73-2013</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>MW-SEG-002</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>Milwaukee</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="inlineStr">
+        <is>
+          <t>Guantes PACKOUT Cut Level 1 Smartswipe</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>48-73-2013</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I49" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="J49" s="18" t="inlineStr">
+        <is>
+          <t>Ver en Milwaukee</t>
+        </is>
+      </c>
+      <c r="K49" s="19" t="inlineStr">
+        <is>
+          <t>https://www.milwaukeetool.com/Search?q=PACKOUT+Cut+Level+Smartswipe+gloves</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="20" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>YN-SEG-001</t>
+        </is>
+      </c>
+      <c r="C50" s="20" t="inlineStr">
+        <is>
+          <t>Youneedthat</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="E50" s="21" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="F50" s="21" t="inlineStr">
+        <is>
+          <t>Guantes aislantes electricos 400V latex (M, 2 pares)</t>
+        </is>
+      </c>
+      <c r="G50" s="20" t="inlineStr">
+        <is>
+          <t>400V-M/2 pairs</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I50" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="J50" s="18" t="inlineStr">
+        <is>
+          <t>Ver en Youneedthat</t>
+        </is>
+      </c>
+      <c r="K50" s="19" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0DSYSKYW2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>MW-ACC-001</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>Milwaukee</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Accesorio</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>Accesorio</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
+        <is>
+          <t>Juego de 3 hojas para Multi-Tool</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>49-10-9001</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I51" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="J51" s="18" t="inlineStr">
+        <is>
+          <t>Ver en Milwaukee</t>
+        </is>
+      </c>
+      <c r="K51" s="19" t="inlineStr">
         <is>
           <t>https://www.milwaukeetool.com/Search?q=49-10-9001</t>
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>MT-ACC-001</t>
+        </is>
+      </c>
+      <c r="C52" s="20" t="inlineStr">
+        <is>
+          <t>MTO</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="inlineStr">
+        <is>
+          <t>Accesorio</t>
+        </is>
+      </c>
+      <c r="E52" s="21" t="inlineStr">
+        <is>
+          <t>Accesorio</t>
+        </is>
+      </c>
+      <c r="F52" s="21" t="inlineStr">
+        <is>
+          <t>Wing Nut Driver Set 4PCS (9/12/15/18mm) 1/4 hex</t>
+        </is>
+      </c>
+      <c r="G52" s="20" t="inlineStr">
+        <is>
+          <t>MTO-WND-4P</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I52" s="17" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+      <c r="J52" s="18" t="inlineStr">
+        <is>
+          <t>Ver en MTO</t>
+        </is>
+      </c>
+      <c r="K52" s="19" t="inlineStr">
+        <is>
+          <t>https://www.amazon.com/dp/B0FD3BHQMV</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:K46"/>
+  <autoFilter ref="A4:K52"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I5:I46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Comprado,Ya tengo"</formula1>
+    <dataValidation sqref="I5:I52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Activo,Baja,Prestado"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -3617,6 +3980,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3657,54 +4032,54 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Prioridad</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Codigo</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>Marca</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>Herramienta</t>
         </is>
       </c>
-      <c r="E4" s="23" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>Modelo</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>Precio (CRC)</t>
         </is>
       </c>
-      <c r="G4" s="23" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
-      <c r="H4" s="23" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Enlace marca</t>
         </is>
       </c>
-      <c r="I4" s="23" t="inlineStr">
+      <c r="I4" s="22" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="n">
+      <c r="A5" s="23" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="15" t="inlineStr">
@@ -3712,40 +4087,40 @@
           <t>KL-SOC-001</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>Klein</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>KNECT 15-Piece Pass Through Socket Set</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="23" t="inlineStr">
         <is>
           <t>65400</t>
         </is>
       </c>
-      <c r="F5" s="25" t="n"/>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>Sockets</t>
         </is>
       </c>
-      <c r="H5" s="26" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>Ver en Klein</t>
         </is>
       </c>
-      <c r="I5" s="27" t="inlineStr">
+      <c r="I5" s="26" t="inlineStr">
         <is>
           <t>https://www.kleintools.com/catalog/socket-wrenches/knect-38-inch-drive-impact-rated-pass-through-socket-set-15-piece</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="n">
+      <c r="A6" s="23" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="15" t="inlineStr">
@@ -3753,42 +4128,42 @@
           <t>KL-MED-001</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>Klein</t>
         </is>
       </c>
-      <c r="D6" s="25" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
         <is>
           <t>Clamp Meter 600A</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="23" t="inlineStr">
         <is>
           <t>CL810</t>
         </is>
       </c>
-      <c r="F6" s="28" t="n">
+      <c r="F6" s="27" t="n">
         <v>80000</v>
       </c>
-      <c r="G6" s="25" t="inlineStr">
+      <c r="G6" s="24" t="inlineStr">
         <is>
           <t>Medicion</t>
         </is>
       </c>
-      <c r="H6" s="26" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
         <is>
           <t>Ver en Klein</t>
         </is>
       </c>
-      <c r="I6" s="27" t="inlineStr">
+      <c r="I6" s="26" t="inlineStr">
         <is>
           <t>https://www.kleintools.com/catalog/clamp-meters/600a-acdc-auto-ranging-trms-clamp-meter-worklight</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="n">
+      <c r="A7" s="23" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="15" t="inlineStr">
@@ -3796,40 +4171,40 @@
           <t>MW-PKO-003</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>Milwaukee</t>
         </is>
       </c>
-      <c r="D7" s="25" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>PACKOUT Rolling Drawer Tool Box</t>
         </is>
       </c>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="E7" s="23" t="inlineStr">
         <is>
           <t>48-22-8420</t>
         </is>
       </c>
-      <c r="F7" s="25" t="n"/>
-      <c r="G7" s="25" t="inlineStr">
+      <c r="F7" s="24" t="n"/>
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>Organizacion</t>
         </is>
       </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="H7" s="25" t="inlineStr">
         <is>
           <t>Ver en Milwaukee</t>
         </is>
       </c>
-      <c r="I7" s="27" t="inlineStr">
+      <c r="I7" s="26" t="inlineStr">
         <is>
           <t>https://www.milwaukeetool.com/Search?q=48-22-8420</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="n">
+      <c r="A8" s="23" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="15" t="inlineStr">
@@ -3837,40 +4212,40 @@
           <t>MW-PKO-004</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>Milwaukee</t>
         </is>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>PACKOUT 2-Wheel Utility Cart</t>
         </is>
       </c>
-      <c r="E8" s="24" t="inlineStr">
+      <c r="E8" s="23" t="inlineStr">
         <is>
           <t>48-22-8415</t>
         </is>
       </c>
-      <c r="F8" s="25" t="n"/>
-      <c r="G8" s="25" t="inlineStr">
+      <c r="F8" s="24" t="n"/>
+      <c r="G8" s="24" t="inlineStr">
         <is>
           <t>Organizacion</t>
         </is>
       </c>
-      <c r="H8" s="26" t="inlineStr">
+      <c r="H8" s="25" t="inlineStr">
         <is>
           <t>Ver en Milwaukee</t>
         </is>
       </c>
-      <c r="I8" s="27" t="inlineStr">
+      <c r="I8" s="26" t="inlineStr">
         <is>
           <t>https://www.milwaukeetool.com/Search?q=48-22-8415</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="n">
+      <c r="A9" s="23" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="15" t="inlineStr">
@@ -3878,42 +4253,42 @@
           <t>MW-M12-008</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>Milwaukee</t>
         </is>
       </c>
-      <c r="D9" s="25" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>M12 AIRSNAKE</t>
         </is>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E9" s="23" t="inlineStr">
         <is>
           <t>2572B-21</t>
         </is>
       </c>
-      <c r="F9" s="28" t="n">
+      <c r="F9" s="27" t="n">
         <v>280000</v>
       </c>
-      <c r="G9" s="25" t="inlineStr">
+      <c r="G9" s="24" t="inlineStr">
         <is>
           <t>Fontaneria</t>
         </is>
       </c>
-      <c r="H9" s="26" t="inlineStr">
+      <c r="H9" s="25" t="inlineStr">
         <is>
           <t>Ver en Milwaukee</t>
         </is>
       </c>
-      <c r="I9" s="27" t="inlineStr">
+      <c r="I9" s="26" t="inlineStr">
         <is>
           <t>https://www.milwaukeetool.com/Search?q=2572B-21</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="n">
+      <c r="A10" s="23" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -3921,45 +4296,45 @@
           <t>CNS-ORD-AMZ-001</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="D10" s="25" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>Terminar de cargar orden consumibles Amazon</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="23" t="inlineStr">
         <is>
           <t>orden haisstronica</t>
         </is>
       </c>
-      <c r="F10" s="25" t="n"/>
-      <c r="G10" s="25" t="inlineStr">
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="24" t="inlineStr">
         <is>
           <t>Consumibles</t>
         </is>
       </c>
-      <c r="H10" s="26" t="inlineStr">
+      <c r="H10" s="25" t="inlineStr">
         <is>
           <t>Ver en Amazon</t>
         </is>
       </c>
-      <c r="I10" s="27" t="inlineStr">
+      <c r="I10" s="26" t="inlineStr">
         <is>
           <t>https://www.amazon.com/</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="E12" s="29" t="inlineStr">
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>Total estimado (con precio):</t>
         </is>
       </c>
-      <c r="F12" s="30">
+      <c r="F12" s="29">
         <f>SUM(F5:F10)</f>
         <v/>
       </c>
@@ -3993,7 +4368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4032,69 +4407,69 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="31" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="31" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Codigo</t>
         </is>
       </c>
-      <c r="C4" s="31" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>Clase</t>
         </is>
       </c>
-      <c r="D4" s="31" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Tipo terminal</t>
         </is>
       </c>
-      <c r="E4" s="31" t="inlineStr">
+      <c r="E4" s="30" t="inlineStr">
         <is>
           <t>Nombre / kit</t>
         </is>
       </c>
-      <c r="F4" s="31" t="inlineStr">
+      <c r="F4" s="30" t="inlineStr">
         <is>
           <t>Marca / ref</t>
         </is>
       </c>
-      <c r="G4" s="31" t="inlineStr">
+      <c r="G4" s="30" t="inlineStr">
         <is>
           <t>Forma</t>
         </is>
       </c>
-      <c r="H4" s="31" t="inlineStr">
+      <c r="H4" s="30" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="I4" s="31" t="inlineStr">
+      <c r="I4" s="30" t="inlineStr">
         <is>
           <t>Umbral reorden</t>
         </is>
       </c>
-      <c r="J4" s="31" t="inlineStr">
+      <c r="J4" s="30" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="K4" s="31" t="inlineStr">
+      <c r="K4" s="30" t="inlineStr">
         <is>
           <t>Ubicacion</t>
         </is>
       </c>
-      <c r="L4" s="31" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Notas / URL</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="32" t="n">
+      <c r="A5" s="31" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="15" t="inlineStr">
@@ -4102,55 +4477,55 @@
           <t>CNS-SPD-ROJ-001</t>
         </is>
       </c>
-      <c r="C5" s="33" t="inlineStr">
+      <c r="C5" s="32" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D5" s="33" t="inlineStr">
+      <c r="D5" s="32" t="inlineStr">
         <is>
           <t>Spade (pala / quick disconnect)</t>
         </is>
       </c>
-      <c r="E5" s="34" t="inlineStr">
+      <c r="E5" s="33" t="inlineStr">
         <is>
           <t>Heat shrink Male/Female — ROJO 22-16 AWG</t>
         </is>
       </c>
-      <c r="F5" s="35" t="inlineStr">
+      <c r="F5" s="34" t="inlineStr">
         <is>
           <t>haisstronica B0D1K6L6TL</t>
         </is>
       </c>
-      <c r="G5" s="32" t="inlineStr">
+      <c r="G5" s="31" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H5" s="32" t="n">
+      <c r="H5" s="31" t="n">
         <v>60</v>
       </c>
-      <c r="I5" s="35" t="n">
+      <c r="I5" s="34" t="n">
         <v>15</v>
       </c>
-      <c r="J5" s="36" t="inlineStr">
+      <c r="J5" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K5" s="37" t="inlineStr">
+      <c r="K5" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L5" s="35" t="inlineStr">
+      <c r="L5" s="34" t="inlineStr">
         <is>
           <t>En PACKOUT Organizer 19 (MW-PKO-005). SPADE rojo. Kit 160PCS. Aprox al reponer.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="n">
+      <c r="A6" s="37" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="15" t="inlineStr">
@@ -4158,55 +4533,55 @@
           <t>CNS-SPD-AZU-001</t>
         </is>
       </c>
-      <c r="C6" s="39" t="inlineStr">
+      <c r="C6" s="38" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D6" s="39" t="inlineStr">
+      <c r="D6" s="38" t="inlineStr">
         <is>
           <t>Spade (pala / quick disconnect)</t>
         </is>
       </c>
-      <c r="E6" s="40" t="inlineStr">
+      <c r="E6" s="39" t="inlineStr">
         <is>
           <t>Heat shrink Male/Female — AZUL 16-14 AWG</t>
         </is>
       </c>
-      <c r="F6" s="41" t="inlineStr">
+      <c r="F6" s="40" t="inlineStr">
         <is>
           <t>haisstronica B0D1K6L6TL</t>
         </is>
       </c>
-      <c r="G6" s="38" t="inlineStr">
+      <c r="G6" s="37" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H6" s="38" t="n">
+      <c r="H6" s="37" t="n">
         <v>60</v>
       </c>
-      <c r="I6" s="41" t="n">
+      <c r="I6" s="40" t="n">
         <v>15</v>
       </c>
-      <c r="J6" s="36" t="inlineStr">
+      <c r="J6" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K6" s="37" t="inlineStr">
+      <c r="K6" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L6" s="41" t="inlineStr">
+      <c r="L6" s="40" t="inlineStr">
         <is>
           <t>En PACKOUT Organizer 19 (MW-PKO-005). SPADE azul. Kit 160PCS. Aprox al reponer.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="42" t="n">
+      <c r="A7" s="41" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="15" t="inlineStr">
@@ -4214,48 +4589,48 @@
           <t>CNS-SPD-AMA-001</t>
         </is>
       </c>
-      <c r="C7" s="43" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D7" s="43" t="inlineStr">
+      <c r="D7" s="42" t="inlineStr">
         <is>
           <t>Spade (pala / quick disconnect)</t>
         </is>
       </c>
-      <c r="E7" s="44" t="inlineStr">
+      <c r="E7" s="43" t="inlineStr">
         <is>
           <t>Heat shrink Male/Female — AMARILLO 12-10 AWG</t>
         </is>
       </c>
-      <c r="F7" s="45" t="inlineStr">
+      <c r="F7" s="44" t="inlineStr">
         <is>
           <t>haisstronica B0D1K6L6TL</t>
         </is>
       </c>
-      <c r="G7" s="42" t="inlineStr">
+      <c r="G7" s="41" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H7" s="42" t="n">
+      <c r="H7" s="41" t="n">
         <v>40</v>
       </c>
-      <c r="I7" s="45" t="n">
+      <c r="I7" s="44" t="n">
         <v>10</v>
       </c>
-      <c r="J7" s="36" t="inlineStr">
+      <c r="J7" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K7" s="37" t="inlineStr">
+      <c r="K7" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L7" s="45" t="inlineStr">
+      <c r="L7" s="44" t="inlineStr">
         <is>
           <t>En PACKOUT Organizer 19 (MW-PKO-005). SPADE amarillo. Kit 160PCS. Aprox al reponer.</t>
         </is>
@@ -4270,17 +4645,17 @@
           <t>CNS-BTT-BLA-001</t>
         </is>
       </c>
-      <c r="C8" s="46" t="inlineStr">
+      <c r="C8" s="45" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D8" s="46" t="inlineStr">
+      <c r="D8" s="45" t="inlineStr">
         <is>
           <t>Butt (empalme / solder seal)</t>
         </is>
       </c>
-      <c r="E8" s="47" t="inlineStr">
+      <c r="E8" s="46" t="inlineStr">
         <is>
           <t>Solder seal butt — BLANCO 26-24 AWG</t>
         </is>
@@ -4301,12 +4676,12 @@
       <c r="I8" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="J8" s="36" t="inlineStr">
+      <c r="J8" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K8" s="37" t="inlineStr">
+      <c r="K8" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
@@ -4318,7 +4693,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="n">
+      <c r="A9" s="31" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="15" t="inlineStr">
@@ -4326,55 +4701,55 @@
           <t>CNS-BTT-ROJ-001</t>
         </is>
       </c>
-      <c r="C9" s="33" t="inlineStr">
+      <c r="C9" s="32" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D9" s="33" t="inlineStr">
+      <c r="D9" s="32" t="inlineStr">
         <is>
           <t>Butt (empalme / solder seal)</t>
         </is>
       </c>
-      <c r="E9" s="34" t="inlineStr">
+      <c r="E9" s="33" t="inlineStr">
         <is>
           <t>Solder seal butt — ROJO 22-18 AWG</t>
         </is>
       </c>
-      <c r="F9" s="35" t="inlineStr">
+      <c r="F9" s="34" t="inlineStr">
         <is>
           <t>haisstronica B07C3NBTJ9</t>
         </is>
       </c>
-      <c r="G9" s="32" t="inlineStr">
+      <c r="G9" s="31" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H9" s="32" t="n">
+      <c r="H9" s="31" t="n">
         <v>45</v>
       </c>
-      <c r="I9" s="35" t="n">
+      <c r="I9" s="34" t="n">
         <v>10</v>
       </c>
-      <c r="J9" s="36" t="inlineStr">
+      <c r="J9" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K9" s="37" t="inlineStr">
+      <c r="K9" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L9" s="35" t="inlineStr">
+      <c r="L9" s="34" t="inlineStr">
         <is>
           <t>Butt solder seal. ROJO 22-18 (0.5-1.0mm2) x45. Kit 120PCS. Ubic. MW-PKO-005.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="38" t="n">
+      <c r="A10" s="37" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -4382,55 +4757,55 @@
           <t>CNS-BTT-AZU-001</t>
         </is>
       </c>
-      <c r="C10" s="39" t="inlineStr">
+      <c r="C10" s="38" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D10" s="39" t="inlineStr">
+      <c r="D10" s="38" t="inlineStr">
         <is>
           <t>Butt (empalme / solder seal)</t>
         </is>
       </c>
-      <c r="E10" s="40" t="inlineStr">
+      <c r="E10" s="39" t="inlineStr">
         <is>
           <t>Solder seal butt — AZUL 16-14 AWG</t>
         </is>
       </c>
-      <c r="F10" s="41" t="inlineStr">
+      <c r="F10" s="40" t="inlineStr">
         <is>
           <t>haisstronica B07C3NBTJ9</t>
         </is>
       </c>
-      <c r="G10" s="38" t="inlineStr">
+      <c r="G10" s="37" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H10" s="38" t="n">
+      <c r="H10" s="37" t="n">
         <v>40</v>
       </c>
-      <c r="I10" s="41" t="n">
+      <c r="I10" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="J10" s="36" t="inlineStr">
+      <c r="J10" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K10" s="37" t="inlineStr">
+      <c r="K10" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L10" s="41" t="inlineStr">
+      <c r="L10" s="40" t="inlineStr">
         <is>
           <t>Butt solder seal. AZUL 16-14 (1.5-2.5mm2) x40. Kit 120PCS. Ubic. MW-PKO-005.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="42" t="n">
+      <c r="A11" s="41" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -4438,48 +4813,48 @@
           <t>CNS-BTT-AMA-001</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="42" t="inlineStr">
         <is>
           <t>Butt (empalme / solder seal)</t>
         </is>
       </c>
-      <c r="E11" s="44" t="inlineStr">
+      <c r="E11" s="43" t="inlineStr">
         <is>
           <t>Solder seal butt — AMARILLO 12-10 AWG</t>
         </is>
       </c>
-      <c r="F11" s="45" t="inlineStr">
+      <c r="F11" s="44" t="inlineStr">
         <is>
           <t>haisstronica B07C3NBTJ9</t>
         </is>
       </c>
-      <c r="G11" s="42" t="inlineStr">
+      <c r="G11" s="41" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H11" s="42" t="n">
+      <c r="H11" s="41" t="n">
         <v>10</v>
       </c>
-      <c r="I11" s="45" t="n">
+      <c r="I11" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="J11" s="36" t="inlineStr">
+      <c r="J11" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K11" s="37" t="inlineStr">
+      <c r="K11" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L11" s="45" t="inlineStr">
+      <c r="L11" s="44" t="inlineStr">
         <is>
           <t>Butt solder seal. AMARILLO 12-10 (4.0-6.0mm2) x10. Kit 120PCS. Ubic. MW-PKO-005.</t>
         </is>
@@ -4494,17 +4869,17 @@
           <t>CNS-BHC-BLA-001</t>
         </is>
       </c>
-      <c r="C12" s="46" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D12" s="46" t="inlineStr">
+      <c r="D12" s="45" t="inlineStr">
         <is>
           <t>Butt (empalme / heat shrink crimp)</t>
         </is>
       </c>
-      <c r="E12" s="47" t="inlineStr">
+      <c r="E12" s="46" t="inlineStr">
         <is>
           <t>Heat shrink crimp butt BHT-0.5 — BLANCO 26-24 AWG (0.5mm)</t>
         </is>
@@ -4525,12 +4900,12 @@
       <c r="I12" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="J12" s="36" t="inlineStr">
+      <c r="J12" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K12" s="37" t="inlineStr">
+      <c r="K12" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
@@ -4542,7 +4917,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="48" t="n">
+      <c r="A13" s="47" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -4550,55 +4925,55 @@
           <t>CNS-BHC-ROS-001</t>
         </is>
       </c>
-      <c r="C13" s="49" t="inlineStr">
+      <c r="C13" s="48" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D13" s="49" t="inlineStr">
+      <c r="D13" s="48" t="inlineStr">
         <is>
           <t>Butt (empalme / heat shrink crimp)</t>
         </is>
       </c>
-      <c r="E13" s="50" t="inlineStr">
+      <c r="E13" s="49" t="inlineStr">
         <is>
           <t>Heat shrink crimp butt BHT-1.25 — ROSA 22-16 AWG (0.7mm)</t>
         </is>
       </c>
-      <c r="F13" s="51" t="inlineStr">
+      <c r="F13" s="50" t="inlineStr">
         <is>
           <t>haisstronica B07RX6QYX5 | BHT-1.25</t>
         </is>
       </c>
-      <c r="G13" s="48" t="inlineStr">
+      <c r="G13" s="47" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H13" s="48" t="n">
+      <c r="H13" s="47" t="n">
         <v>50</v>
       </c>
-      <c r="I13" s="51" t="n">
+      <c r="I13" s="50" t="n">
         <v>12</v>
       </c>
-      <c r="J13" s="36" t="inlineStr">
+      <c r="J13" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K13" s="37" t="inlineStr">
+      <c r="K13" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L13" s="51" t="inlineStr">
+      <c r="L13" s="50" t="inlineStr">
         <is>
           <t>Butt heat-shrink CRIMP. BHT-1.25 rosa/pink (a veces listado rojo). Kit 200PCS. Ubic. MW-PKO-005.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="38" t="n">
+      <c r="A14" s="37" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="15" t="inlineStr">
@@ -4606,55 +4981,55 @@
           <t>CNS-BHC-AZU-001</t>
         </is>
       </c>
-      <c r="C14" s="39" t="inlineStr">
+      <c r="C14" s="38" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D14" s="39" t="inlineStr">
+      <c r="D14" s="38" t="inlineStr">
         <is>
           <t>Butt (empalme / heat shrink crimp)</t>
         </is>
       </c>
-      <c r="E14" s="40" t="inlineStr">
+      <c r="E14" s="39" t="inlineStr">
         <is>
           <t>Heat shrink crimp butt BHT-2 — AZUL 16-14 AWG (0.8mm)</t>
         </is>
       </c>
-      <c r="F14" s="41" t="inlineStr">
+      <c r="F14" s="40" t="inlineStr">
         <is>
           <t>haisstronica B07RX6QYX5 | BHT-2</t>
         </is>
       </c>
-      <c r="G14" s="38" t="inlineStr">
+      <c r="G14" s="37" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H14" s="38" t="n">
+      <c r="H14" s="37" t="n">
         <v>50</v>
       </c>
-      <c r="I14" s="41" t="n">
+      <c r="I14" s="40" t="n">
         <v>12</v>
       </c>
-      <c r="J14" s="36" t="inlineStr">
+      <c r="J14" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K14" s="37" t="inlineStr">
+      <c r="K14" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L14" s="41" t="inlineStr">
+      <c r="L14" s="40" t="inlineStr">
         <is>
           <t>Butt heat-shrink CRIMP. BHT-2 azul. Kit 200PCS. Ubic. MW-PKO-005.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="42" t="n">
+      <c r="A15" s="41" t="n">
         <v>11</v>
       </c>
       <c r="B15" s="15" t="inlineStr">
@@ -4662,55 +5037,55 @@
           <t>CNS-BHC-AMA-001</t>
         </is>
       </c>
-      <c r="C15" s="43" t="inlineStr">
+      <c r="C15" s="42" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>Butt (empalme / heat shrink crimp)</t>
         </is>
       </c>
-      <c r="E15" s="44" t="inlineStr">
+      <c r="E15" s="43" t="inlineStr">
         <is>
           <t>Heat shrink crimp butt BHT-5.5 — AMARILLO 12-10 AWG (1.0mm)</t>
         </is>
       </c>
-      <c r="F15" s="45" t="inlineStr">
+      <c r="F15" s="44" t="inlineStr">
         <is>
           <t>haisstronica B07RX6QYX5 | BHT-5.5</t>
         </is>
       </c>
-      <c r="G15" s="42" t="inlineStr">
+      <c r="G15" s="41" t="inlineStr">
         <is>
           <t>aprox</t>
         </is>
       </c>
-      <c r="H15" s="42" t="n">
+      <c r="H15" s="41" t="n">
         <v>50</v>
       </c>
-      <c r="I15" s="45" t="n">
+      <c r="I15" s="44" t="n">
         <v>12</v>
       </c>
-      <c r="J15" s="36" t="inlineStr">
+      <c r="J15" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K15" s="37" t="inlineStr">
+      <c r="K15" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L15" s="45" t="inlineStr">
+      <c r="L15" s="44" t="inlineStr">
         <is>
           <t>Butt heat-shrink CRIMP. BHT-5.5 amarillo. Kit 200PCS. Ubic. MW-PKO-005.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="52" t="n">
+      <c r="A16" s="51" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="15" t="inlineStr">
@@ -4718,109 +5093,221 @@
           <t>CNS-BNI-1210-001</t>
         </is>
       </c>
-      <c r="C16" s="53" t="inlineStr">
+      <c r="C16" s="52" t="inlineStr">
         <is>
           <t>Conector electrico</t>
         </is>
       </c>
-      <c r="D16" s="53" t="inlineStr">
+      <c r="D16" s="52" t="inlineStr">
         <is>
           <t>Butt (empalme / non-insulated crimp)</t>
         </is>
       </c>
-      <c r="E16" s="54" t="inlineStr">
+      <c r="E16" s="53" t="inlineStr">
         <is>
           <t>Non-insulated butt tinned copper — AWG 12-10 (50PCS)</t>
         </is>
       </c>
-      <c r="F16" s="55" t="inlineStr">
+      <c r="F16" s="54" t="inlineStr">
         <is>
           <t>haisstronica B0F1N2WH51</t>
         </is>
       </c>
-      <c r="G16" s="52" t="inlineStr">
+      <c r="G16" s="51" t="inlineStr">
         <is>
           <t>paquete</t>
         </is>
       </c>
-      <c r="H16" s="52" t="n">
+      <c r="H16" s="51" t="n">
         <v>50</v>
       </c>
-      <c r="I16" s="55" t="n">
+      <c r="I16" s="54" t="n">
         <v>12</v>
       </c>
-      <c r="J16" s="36" t="inlineStr">
+      <c r="J16" s="35" t="inlineStr">
         <is>
           <t>Tengo</t>
         </is>
       </c>
-      <c r="K16" s="37" t="inlineStr">
+      <c r="K16" s="36" t="inlineStr">
         <is>
           <t>MW-PKO-005</t>
         </is>
       </c>
-      <c r="L16" s="55" t="inlineStr">
+      <c r="L16" s="54" t="inlineStr">
         <is>
           <t>Butt NO aislado, cobre estanado. Solo 12-10 AWG x50. Recomienda heat shrink aparte. Ubic. MW-PKO-005.</t>
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="51" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>CNS-RNI-516-001</t>
+        </is>
+      </c>
+      <c r="C17" s="52" t="inlineStr">
+        <is>
+          <t>Conector electrico</t>
+        </is>
+      </c>
+      <c r="D17" s="52" t="inlineStr">
+        <is>
+          <t>Ring (ojal / non-insulated crimp)</t>
+        </is>
+      </c>
+      <c r="E17" s="53" t="inlineStr">
+        <is>
+          <t>Kit ring 5/16" stud AWG 12-10 + heat shrink 3:1 (50+50)</t>
+        </is>
+      </c>
+      <c r="F17" s="54" t="inlineStr">
+        <is>
+          <t>haisstronica B0F2T8LR9W</t>
+        </is>
+      </c>
+      <c r="G17" s="51" t="inlineStr">
+        <is>
+          <t>paquete</t>
+        </is>
+      </c>
+      <c r="H17" s="51" t="n">
+        <v>50</v>
+      </c>
+      <c r="I17" s="54" t="n">
+        <v>12</v>
+      </c>
+      <c r="J17" s="35" t="inlineStr">
+        <is>
+          <t>Tengo</t>
+        </is>
+      </c>
+      <c r="K17" s="36" t="inlineStr">
+        <is>
+          <t>MW-PKO-005</t>
+        </is>
+      </c>
+      <c r="L17" s="54" t="inlineStr">
+        <is>
+          <t>Ring NO aislado 5/16 stud, cobre estanado, brazed seam x50 + 50 tubos 3:1 rojo/negro. Ubic. MW-PKO-005.</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="51" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>CNS-FNI-10-001</t>
+        </is>
+      </c>
+      <c r="C18" s="52" t="inlineStr">
+        <is>
+          <t>Conector electrico</t>
+        </is>
+      </c>
+      <c r="D18" s="52" t="inlineStr">
+        <is>
+          <t>Fork (horquilla / non-insulated crimp)</t>
+        </is>
+      </c>
+      <c r="E18" s="53" t="inlineStr">
+        <is>
+          <t>Kit fork #10 stud AWG 12-10 + heat shrink 3:1 (50+50)</t>
+        </is>
+      </c>
+      <c r="F18" s="54" t="inlineStr">
+        <is>
+          <t>haisstronica B0F2T498YF</t>
+        </is>
+      </c>
+      <c r="G18" s="51" t="inlineStr">
+        <is>
+          <t>paquete</t>
+        </is>
+      </c>
+      <c r="H18" s="51" t="n">
+        <v>50</v>
+      </c>
+      <c r="I18" s="54" t="n">
+        <v>12</v>
+      </c>
+      <c r="J18" s="35" t="inlineStr">
+        <is>
+          <t>Tengo</t>
+        </is>
+      </c>
+      <c r="K18" s="36" t="inlineStr">
+        <is>
+          <t>MW-PKO-005</t>
+        </is>
+      </c>
+      <c r="L18" s="54" t="inlineStr">
+        <is>
+          <t>Fork NO aislado #10 stud, cobre estanado, brazed seam x50 + 50 tubos 3:1 rojo/negro. Ubic. MW-PKO-005.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Como usar:</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="56" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="55" t="inlineStr">
         <is>
           <t>1) Clase = familia (Conector electrico, Cinta / aislante, Fijacion...).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="56" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="55" t="inlineStr">
         <is>
           <t>2) Tipo terminal solo si Clase=Conector electrico; si no, '—'.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="56" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="55" t="inlineStr">
         <is>
           <t>3) Ubicacion = codigo del contenedor (MW-PKO-005 = Organizer 19 pulg PACKOUT).</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="56" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="55" t="inlineStr">
         <is>
           <t>4) Por COLOR en filas. Reponer si baja umbral. Clic en Nombre (col E) = link.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L16"/>
+  <autoFilter ref="A4:L18"/>
   <mergeCells count="3">
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="J5:J16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J5:J18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Tengo,Reponer"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G5:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"kit,paquete,aprox"</formula1>
     </dataValidation>
-    <dataValidation sqref="C5:C16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C5:C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Conector electrico,Cinta / aislante,Fijacion,Corte / desgaste,Quimico / sellado,Otro"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Spade (pala / quick disconnect),Butt (empalme / solder seal),Butt (empalme / heat shrink crimp),Butt (empalme / non-insulated crimp),Ring (anillo),Fork (horquilla),Wire nut,—,Otro"</formula1>
     </dataValidation>
-    <dataValidation sqref="K5:K16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"MW-PKO-001,MW-PKO-002,MW-PKO-005,MW-PKO-003,MW-PKO-004,Taller,Vehiculo,Otro"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4837,6 +5324,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>